<commit_message>
Add seed rotation, overnight breakfasts and YouTube recipe references
</commit_message>
<xml_diff>
--- a/downloads/shopping_list_all_vitamins.xlsx
+++ b/downloads/shopping_list_all_vitamins.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costco Wesley Chapel" sheetId="1" r:id="R7b6ec189190649ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Walmart Wesley Chapel" sheetId="2" r:id="Rdda4c60f7f364b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Store Comparison" sheetId="3" r:id="Rf4fc52d3320e4a23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Sources" sheetId="4" r:id="R0abb52fa28824ce6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lotte Tampa" sheetId="5" r:id="Rb96fa3a141ee4f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitamin Coverage" sheetId="6" r:id="R6ec3d50aa8ec4065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitamin Targets" sheetId="7" r:id="R6b6aca25323b4bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costco Wesley Chapel" sheetId="1" r:id="Rc7d315346b3b4f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Walmart Wesley Chapel" sheetId="2" r:id="Rd9c2c56ff2524ff1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Store Comparison" sheetId="3" r:id="Racf5d4db5cd2496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Sources" sheetId="4" r:id="Rcf49efba84e940a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lotte Tampa" sheetId="5" r:id="Rb2d93f57d05f4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitamin Coverage" sheetId="6" r:id="Rfa3cd6044e4c4c2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitamin Targets" sheetId="7" r:id="R107462b5c4fb451c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Breakfast Flex Shopping" sheetId="8" r:id="R9693670086ac43f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -30,8 +31,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -68,6 +74,36 @@
         <x:fgColor rgb="FF548235"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF70AD47"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF548235"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFA9D18E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B9BD5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -76,7 +112,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -143,6 +179,44 @@
     <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -237,7 +311,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -247,7 +321,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -257,7 +331,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -267,7 +341,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -277,7 +351,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -287,7 +361,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -297,7 +371,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -307,7 +381,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -317,7 +391,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -327,7 +401,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -337,7 +411,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -347,7 +421,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -357,7 +431,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -367,7 +441,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -377,7 +451,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -387,7 +461,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -397,7 +471,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -407,7 +481,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -417,7 +491,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -427,7 +501,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -437,7 +511,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -447,7 +521,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -457,7 +531,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -467,7 +541,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -477,7 +551,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -487,7 +561,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -497,7 +571,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -507,7 +581,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -517,7 +591,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -527,7 +601,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -537,7 +611,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -547,7 +621,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -557,7 +631,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -567,7 +641,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -577,7 +651,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -587,7 +661,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -597,7 +671,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -607,7 +681,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -617,7 +691,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -1743,7 +1817,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f41828c5ded4bb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48de0586c9114fc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2583,7 +2657,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5899d0f9ecb34ddb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae23659bffbf48d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2592,39 +2666,39 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="19" t="str">
+      <x:c r="A1" s="32" t="str">
         <x:v>Department</x:v>
       </x:c>
-      <x:c r="B1" s="19" t="str">
+      <x:c r="B1" s="32" t="str">
         <x:v>Item</x:v>
       </x:c>
-      <x:c r="C1" s="19" t="str">
+      <x:c r="C1" s="32" t="str">
         <x:v>Weekly Need</x:v>
       </x:c>
-      <x:c r="D1" s="19" t="str">
+      <x:c r="D1" s="32" t="str">
         <x:v>Costco Wesley Chapel</x:v>
       </x:c>
-      <x:c r="E1" s="19" t="str">
+      <x:c r="E1" s="32" t="str">
         <x:v>Walmart Wesley Chapel</x:v>
       </x:c>
-      <x:c r="F1" s="19" t="str">
+      <x:c r="F1" s="32" t="str">
         <x:v>Lotte Tampa</x:v>
       </x:c>
-      <x:c r="G1" s="19" t="str">
+      <x:c r="G1" s="32" t="str">
         <x:v>Recommended Store</x:v>
       </x:c>
-      <x:c r="H1" s="19" t="str">
+      <x:c r="H1" s="32" t="str">
         <x:v>Why</x:v>
       </x:c>
     </x:row>
@@ -3078,7 +3152,7 @@
         <x:v>Rolled oats</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>225 g</x:v>
+        <x:v>194 g</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
         <x:v>1 bulk bag</x:v>
@@ -3093,7 +3167,7 @@
         <x:v>Walmart</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
-        <x:v>Smaller conventional package better matches the one-week requirement.</x:v>
+        <x:v>Recommended Option 1 now uses 194 g/week; a smaller conventional package minimizes waste.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3145,7 +3219,7 @@
         <x:v>Lotte</x:v>
       </x:c>
       <x:c r="H21" s="12" t="str">
-        <x:v>Frequent ragi use remains in the final plan; Lotte/Indian grocery is the better category fit.</x:v>
+        <x:v>Base plan still uses cooked ragi flour 180 g/week. Raw ragi flour is not used in no-cook overnight jars.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -3286,7 +3360,7 @@
         <x:v>Sesame seeds</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>174 g</x:v>
+        <x:v>164 g</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
         <x:v>Bulk only if frequently used</x:v>
@@ -3301,7 +3375,7 @@
         <x:v>Lotte</x:v>
       </x:c>
       <x:c r="H27" s="12" t="str">
-        <x:v>Final weekly need rose to 174 g; Lotte is a strong fit for a practical sesame package.</x:v>
+        <x:v>Revised breakfast rotation reduces weekly sesame to 164 g while retaining sesame in lunches/dinners.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -3312,7 +3386,7 @@
         <x:v>Ground flaxseed</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>35 g</x:v>
+        <x:v>17 g</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
         <x:v>Bulk bag if regularly used</x:v>
@@ -3327,7 +3401,7 @@
         <x:v>Walmart</x:v>
       </x:c>
       <x:c r="H28" s="12" t="str">
-        <x:v>Final weekly need is 35 g; smaller package minimizes waste.</x:v>
+        <x:v>Revised breakfast seed rotation uses 17 g/week in the recommended Option 1 schedule.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -3338,7 +3412,7 @@
         <x:v>Chia seeds</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>32 g</x:v>
+        <x:v>33 g</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
         <x:v>Bulk bag if regularly used</x:v>
@@ -3353,110 +3427,188 @@
         <x:v>Walmart</x:v>
       </x:c>
       <x:c r="H29" s="12" t="str">
-        <x:v>Final weekly need is 32 g after adding 5 g on Day 2 to close the omega-3 planning gap.</x:v>
+        <x:v>Revised breakfast seed rotation uses 33 g/week in the recommended Option 1 schedule.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="12" t="str">
-        <x:v>Frozen</x:v>
+        <x:v>Pantry &amp; Dry Goods</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>Frozen sweet peas</x:v>
+        <x:v>Hemp hearts</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>300 g</x:v>
+        <x:v>20 g</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>1 bulk frozen bag if stocked</x:v>
+        <x:v>Large bag if stocked; excess for one week</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>1 × 12–16 oz bag</x:v>
+        <x:v>1 small bag/pouch</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>1 small/medium frozen bag</x:v>
+        <x:v>Check health/international aisle</x:v>
       </x:c>
       <x:c r="G30" s="12" t="str">
         <x:v>Walmart</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
-        <x:v>Smaller conventional package better matches the one-week requirement.</x:v>
+        <x:v>Only 20 g/week is needed in the base breakfast rotation; smaller packaging is more practical.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="12" t="str">
-        <x:v>Seafood / Specialty</x:v>
+        <x:v>Pantry &amp; Dry Goods</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>ICAN Icelandic Wild Cod Liver</x:v>
+        <x:v>Pumpkin seeds / pepitas</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>20 g</x:v>
+        <x:v>10 g</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>Not standard Costco inventory</x:v>
+        <x:v>Large bag; significant excess</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>1 × 115 g can / online if available</x:v>
+        <x:v>1 small bag</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>Not confirmed; use Walmart/online product</x:v>
+        <x:v>1 small bag; verify</x:v>
       </x:c>
       <x:c r="G31" s="12" t="str">
         <x:v>Walmart</x:v>
       </x:c>
       <x:c r="H31" s="12" t="str">
-        <x:v>Smaller conventional package better matches the one-week requirement.</x:v>
+        <x:v>Only 10 g/week is needed in the base breakfast rotation; buy unsalted/plain.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="12" t="str">
-        <x:v>Seafood</x:v>
+        <x:v>Pantry &amp; Dry Goods</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>Tilapia fillet</x:v>
+        <x:v>Sunflower seeds</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>160 g</x:v>
+        <x:v>20 g</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>Not planned</x:v>
+        <x:v>Large bag; significant excess</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>Not planned</x:v>
+        <x:v>1 small bag</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>~1 lb sale pack at $4.99/lb</x:v>
+        <x:v>1 small bag; verify</x:v>
       </x:c>
       <x:c r="G32" s="12" t="str">
-        <x:v>Lotte</x:v>
+        <x:v>Walmart</x:v>
       </x:c>
       <x:c r="H32" s="12" t="str">
-        <x:v>One 160 g fish meal; FDA/EPA Best Choice for mercury.</x:v>
+        <x:v>Added mainly for breakfast variety and vitamin E exposure; buy plain/unsalted.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="12" t="str">
+        <x:v>Frozen</x:v>
+      </x:c>
+      <x:c r="B33" s="12" t="str">
+        <x:v>Frozen sweet peas</x:v>
+      </x:c>
+      <x:c r="C33" s="12" t="str">
+        <x:v>300 g</x:v>
+      </x:c>
+      <x:c r="D33" s="12" t="str">
+        <x:v>1 bulk frozen bag if stocked</x:v>
+      </x:c>
+      <x:c r="E33" s="12" t="str">
+        <x:v>1 × 12–16 oz bag</x:v>
+      </x:c>
+      <x:c r="F33" s="12" t="str">
+        <x:v>1 small/medium frozen bag</x:v>
+      </x:c>
+      <x:c r="G33" s="12" t="str">
+        <x:v>Walmart</x:v>
+      </x:c>
+      <x:c r="H33" s="12" t="str">
+        <x:v>Smaller conventional package better matches the one-week requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="12" t="str">
+        <x:v>Seafood / Specialty</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>ICAN Icelandic Wild Cod Liver</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str">
+        <x:v>20 g</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="str">
+        <x:v>Not standard Costco inventory</x:v>
+      </x:c>
+      <x:c r="E34" s="12" t="str">
+        <x:v>1 × 115 g can / online if available</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="str">
+        <x:v>Not confirmed; use Walmart/online product</x:v>
+      </x:c>
+      <x:c r="G34" s="12" t="str">
+        <x:v>Walmart</x:v>
+      </x:c>
+      <x:c r="H34" s="12" t="str">
+        <x:v>Smaller conventional package better matches the one-week requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="12" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="B33" s="12" t="str">
+      <x:c r="B35" s="12" t="str">
+        <x:v>Tilapia fillet</x:v>
+      </x:c>
+      <x:c r="C35" s="12" t="str">
+        <x:v>160 g</x:v>
+      </x:c>
+      <x:c r="D35" s="12" t="str">
+        <x:v>Not planned</x:v>
+      </x:c>
+      <x:c r="E35" s="12" t="str">
+        <x:v>Not planned</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="str">
+        <x:v>~1 lb sale pack at $4.99/lb</x:v>
+      </x:c>
+      <x:c r="G35" s="12" t="str">
+        <x:v>Lotte</x:v>
+      </x:c>
+      <x:c r="H35" s="12" t="str">
+        <x:v>One 160 g fish meal; FDA/EPA Best Choice for mercury.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="12" t="str">
+        <x:v>Seafood</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
         <x:v>Ocean perch fillet</x:v>
       </x:c>
-      <x:c r="C33" s="12" t="str">
+      <x:c r="C36" s="12" t="str">
         <x:v>160 g</x:v>
       </x:c>
-      <x:c r="D33" s="12" t="str">
+      <x:c r="D36" s="12" t="str">
         <x:v>Not planned</x:v>
       </x:c>
-      <x:c r="E33" s="12" t="str">
+      <x:c r="E36" s="12" t="str">
         <x:v>Not planned</x:v>
       </x:c>
-      <x:c r="F33" s="12" t="str">
+      <x:c r="F36" s="12" t="str">
         <x:v>~1 lb sale pack at $4.99/lb</x:v>
       </x:c>
-      <x:c r="G33" s="12" t="str">
+      <x:c r="G36" s="12" t="str">
         <x:v>Lotte</x:v>
       </x:c>
-      <x:c r="H33" s="12" t="str">
+      <x:c r="H36" s="12" t="str">
         <x:v>One 160 g fish meal; FDA/EPA Best Choice for mercury.</x:v>
       </x:c>
     </x:row>
@@ -3488,8 +3640,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92aa3f85a2fe4a33"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd468ca33a7034b84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R143a641438764e2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfec0edc86759470d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3498,17 +3650,18 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="95" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="20" t="str">
+      <x:c r="A1" s="47" t="str">
         <x:v>Topic</x:v>
       </x:c>
-      <x:c r="B1" s="20" t="str">
+      <x:c r="B1" s="47" t="str">
         <x:v>Details</x:v>
       </x:c>
+      <x:c r="C1" s="46"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="12" t="str">
@@ -3517,6 +3670,7 @@
       <x:c r="B2" s="12" t="str">
         <x:v>Costco Wesley Chapel Warehouse #1249, 2225 Grand Cypress Dr, Lutz, FL 33559.</x:v>
       </x:c>
+      <x:c r="C2" s="12"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="12" t="str">
@@ -3525,6 +3679,7 @@
       <x:c r="B3" s="12" t="str">
         <x:v>Walmart Supercenter #3418, 28500 State Road 54, Wesley Chapel, FL 33543.</x:v>
       </x:c>
+      <x:c r="C3" s="12"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="12" t="str">
@@ -3533,6 +3688,7 @@
       <x:c r="B4" s="12" t="str">
         <x:v>17605 Bruce B Downs Blvd, Tampa, FL 33647.</x:v>
       </x:c>
+      <x:c r="C4" s="12"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="12" t="str">
@@ -3541,14 +3697,16 @@
       <x:c r="B5" s="12" t="str">
         <x:v>Fresh inventory and package sizes change; verify current stock in the relevant store/app before the trip.</x:v>
       </x:c>
+      <x:c r="C5" s="12"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="12" t="str">
         <x:v>Meal-plan basis</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Synchronized to the final verified 7-day plan: 1,700–1,900 kcal/day; protein 110–130 g/day; frequent ragi; no tofu/salmon; tilapia 160 g + ocean perch 160 g; cod liver 20 g once weekly; no curd/yogurt in the final plan.</x:v>
-      </x:c>
+        <x:v>Synchronized to the approved breakfast-seed/overnight revision: 1,700–1,900 kcal/day; protein 110–130 g/day; 4 breakfast options/day; Option 4 is no-cook in the morning; frequent ragi; no tofu/salmon; tilapia 160 g + ocean perch 160 g; cod liver 20 g once weekly.</x:v>
+      </x:c>
+      <x:c r="C6" s="12"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="12" t="str">
@@ -3557,6 +3715,7 @@
       <x:c r="B7" s="12" t="str">
         <x:v>Fruit is separate; milk breakfasts contain no added salt/onion/garlic; chicken/fish/goat meals contain no dairy.</x:v>
       </x:c>
+      <x:c r="C7" s="12"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="12" t="str">
@@ -3565,6 +3724,7 @@
       <x:c r="B8" s="12" t="str">
         <x:v>Cooking oil and negligible-quantity basic seasonings are omitted from this shopping checklist.</x:v>
       </x:c>
+      <x:c r="C8" s="12"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="12" t="str">
@@ -3573,6 +3733,7 @@
       <x:c r="B9" s="12" t="str">
         <x:v>https://www.ewg.org/foodnews/dirty-dozen.php</x:v>
       </x:c>
+      <x:c r="C9" s="12"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="12" t="str">
@@ -3581,6 +3742,7 @@
       <x:c r="B10" s="12" t="str">
         <x:v>https://www.ewg.org/foodnews/full-list.php</x:v>
       </x:c>
+      <x:c r="C10" s="12"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="12" t="str">
@@ -3589,6 +3751,7 @@
       <x:c r="B11" s="12" t="str">
         <x:v>https://www.fda.gov/food/consumers/advice-about-eating-fish</x:v>
       </x:c>
+      <x:c r="C11" s="12"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="12" t="str">
@@ -3597,6 +3760,7 @@
       <x:c r="B12" s="12" t="str">
         <x:v>FDA/EPA lists tilapia and perch (freshwater and ocean) as Best Choices for mercury.</x:v>
       </x:c>
+      <x:c r="C12" s="12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
@@ -3605,6 +3769,7 @@
       <x:c r="B13" s="12" t="str">
         <x:v>User-supplied flyer: tilapia fillet $4.99/lb and ocean perch fillet $4.99/lb.</x:v>
       </x:c>
+      <x:c r="C13" s="12"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="12" t="str">
@@ -3613,6 +3778,7 @@
       <x:c r="B14" s="12" t="str">
         <x:v>Buy/portion 160 g tilapia for Day 4 and 160 g ocean perch for Day 6; freeze unused sale-pack portions promptly.</x:v>
       </x:c>
+      <x:c r="C14" s="12"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="12" t="str">
@@ -3621,6 +3787,7 @@
       <x:c r="B15" s="12" t="str">
         <x:v>Final weekly chicken need is 800 g and lean goat/mutton 100 g after rebalancing to 110–130 g/day protein.</x:v>
       </x:c>
+      <x:c r="C15" s="12"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="12" t="str">
@@ -3629,14 +3796,16 @@
       <x:c r="B16" s="12" t="str">
         <x:v>Greek yogurt/curd is no longer used. Low-fat milk requirement is 2,100 ml/week.</x:v>
       </x:c>
+      <x:c r="C16" s="12"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="12" t="str">
-        <x:v>Omega-3 seed update</x:v>
+        <x:v>Breakfast seed rotation</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Ground flaxseed need is 35 g/week; chia need is 32 g/week; sesame need is 174 g/week.</x:v>
-      </x:c>
+        <x:v>Recommended Option 1 weekly base: chia 33 g, ground flax 17 g, hemp hearts 20 g, pumpkin seeds 10 g, sunflower seeds 20 g; sesame total 164 g including all meals.</x:v>
+      </x:c>
+      <x:c r="C17" s="12"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="12" t="str">
@@ -3645,14 +3814,43 @@
       <x:c r="B18" s="12" t="str">
         <x:v>This shopping workbook now includes the same Daily Nutrition vitamin panel as the final meal-plan workbook: A, C, D, E, K, B1, B2, B3, B5, B6, B7, B9 and B12, plus preformed vitamin A.</x:v>
       </x:c>
+      <x:c r="C18" s="12"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="12" t="str">
         <x:v>Shopping quantity impact</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>Adding vitamin tracking did not change the final ingredient quantities; Vitamin Coverage is informational only.</x:v>
-      </x:c>
+        <x:v>Main Store Comparison is based on recommended Breakfast Option 1. Use Breakfast Flex Shopping for optional Option 2–4 ingredients; do not buy every alternative ingredient unless you plan to use it.</x:v>
+      </x:c>
+      <x:c r="C19" s="12"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="12" t="str">
+        <x:v>Overnight shopping</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>If using Option 4, buy rolled oats / thick poha / label-confirmed ready-to-eat or steam-processed ragi flakes according to the days selected. Raw ragi flour is not a no-cook substitute.</x:v>
+      </x:c>
+      <x:c r="C20" s="12"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="12" t="str">
+        <x:v>Seed handling</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>Breakfast seeds are measured and eaten as a separate side, not stirred into the milk/grain bowl. Buy plain/unsalted seeds.</x:v>
+      </x:c>
+      <x:c r="C21" s="12"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="12" t="str">
+        <x:v>YouTube references</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>Recipe videos are stored in the meal-plan workbook and are technique references only; workbook quantities/rules override external videos.</x:v>
+      </x:c>
+      <x:c r="C22" s="12"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4495,7 +4693,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3fd9b6e699644f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ac77a2ca6e140af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4533,82 +4731,82 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="25" t="str">
+      <x:c r="A1" s="45" t="str">
         <x:v>Day</x:v>
       </x:c>
-      <x:c r="B1" s="25" t="str">
+      <x:c r="B1" s="45" t="str">
         <x:v>Calories</x:v>
       </x:c>
-      <x:c r="C1" s="25" t="str">
+      <x:c r="C1" s="45" t="str">
         <x:v>Protein g</x:v>
       </x:c>
-      <x:c r="D1" s="25" t="str">
+      <x:c r="D1" s="45" t="str">
         <x:v>Carbs g</x:v>
       </x:c>
-      <x:c r="E1" s="25" t="str">
+      <x:c r="E1" s="45" t="str">
         <x:v>Fiber g</x:v>
       </x:c>
-      <x:c r="F1" s="25" t="str">
+      <x:c r="F1" s="45" t="str">
         <x:v>Fat g</x:v>
       </x:c>
-      <x:c r="G1" s="25" t="str">
+      <x:c r="G1" s="45" t="str">
         <x:v>Calcium mg</x:v>
       </x:c>
-      <x:c r="H1" s="25" t="str">
+      <x:c r="H1" s="45" t="str">
         <x:v>Iron mg</x:v>
       </x:c>
-      <x:c r="I1" s="25" t="str">
+      <x:c r="I1" s="45" t="str">
         <x:v>Magnesium mg</x:v>
       </x:c>
-      <x:c r="J1" s="25" t="str">
+      <x:c r="J1" s="45" t="str">
         <x:v>Potassium mg</x:v>
       </x:c>
-      <x:c r="K1" s="25" t="str">
+      <x:c r="K1" s="45" t="str">
         <x:v>Vitamin B12 (µg)</x:v>
       </x:c>
-      <x:c r="L1" s="25" t="str">
+      <x:c r="L1" s="45" t="str">
         <x:v>Vitamin D (µg)</x:v>
       </x:c>
-      <x:c r="M1" s="25" t="str">
+      <x:c r="M1" s="45" t="str">
         <x:v>Vitamin B9 Folate (µg DFE)</x:v>
       </x:c>
-      <x:c r="N1" s="25" t="str">
+      <x:c r="N1" s="45" t="str">
         <x:v>Omega-3 (g)</x:v>
       </x:c>
-      <x:c r="O1" s="25" t="str">
+      <x:c r="O1" s="45" t="str">
         <x:v>Saturated Fat (g)</x:v>
       </x:c>
-      <x:c r="P1" s="25" t="str">
+      <x:c r="P1" s="45" t="str">
         <x:v>Preformed Vitamin A (µg RAE)</x:v>
       </x:c>
-      <x:c r="Q1" s="25" t="str">
+      <x:c r="Q1" s="45" t="str">
         <x:v>Vitamin A Total (µg RAE)</x:v>
       </x:c>
-      <x:c r="R1" s="25" t="str">
+      <x:c r="R1" s="45" t="str">
         <x:v>Vitamin C (mg)</x:v>
       </x:c>
-      <x:c r="S1" s="25" t="str">
+      <x:c r="S1" s="45" t="str">
         <x:v>Vitamin E (mg)</x:v>
       </x:c>
-      <x:c r="T1" s="25" t="str">
+      <x:c r="T1" s="45" t="str">
         <x:v>Vitamin K (µg)</x:v>
       </x:c>
-      <x:c r="U1" s="25" t="str">
+      <x:c r="U1" s="45" t="str">
         <x:v>Vitamin B1 Thiamin (mg)</x:v>
       </x:c>
-      <x:c r="V1" s="25" t="str">
+      <x:c r="V1" s="45" t="str">
         <x:v>Vitamin B2 Riboflavin (mg)</x:v>
       </x:c>
-      <x:c r="W1" s="25" t="str">
+      <x:c r="W1" s="45" t="str">
         <x:v>Vitamin B3 Niacin (mg)</x:v>
       </x:c>
-      <x:c r="X1" s="25" t="str">
+      <x:c r="X1" s="45" t="str">
         <x:v>Vitamin B5 Pantothenic Acid (mg)</x:v>
       </x:c>
-      <x:c r="Y1" s="25" t="str">
+      <x:c r="Y1" s="45" t="str">
         <x:v>Vitamin B6 (mg)</x:v>
       </x:c>
-      <x:c r="Z1" s="25" t="str">
+      <x:c r="Z1" s="45" t="str">
         <x:v>Vitamin B7 Biotin (µg, est.)</x:v>
       </x:c>
     </x:row>
@@ -4617,79 +4815,79 @@
         <x:v>Day 1</x:v>
       </x:c>
       <x:c r="B2" s="12" t="n">
-        <x:v>1756.4</x:v>
+        <x:v>1772.9</x:v>
       </x:c>
       <x:c r="C2" s="12" t="n">
-        <x:v>119.1</x:v>
+        <x:v>120.3</x:v>
       </x:c>
       <x:c r="D2" s="12" t="n">
-        <x:v>212.79999999999998</x:v>
+        <x:v>212.8</x:v>
       </x:c>
       <x:c r="E2" s="12" t="n">
-        <x:v>38.5</x:v>
+        <x:v>38.2</x:v>
       </x:c>
       <x:c r="F2" s="12" t="n">
-        <x:v>51.599999999999994</x:v>
+        <x:v>53.1</x:v>
       </x:c>
       <x:c r="G2" s="12" t="n">
-        <x:v>1007.1000000000001</x:v>
+        <x:v>1009.3</x:v>
       </x:c>
       <x:c r="H2" s="12" t="n">
-        <x:v>16.7</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I2" s="12" t="n">
-        <x:v>533.1</x:v>
+        <x:v>559.7</x:v>
       </x:c>
       <x:c r="J2" s="12" t="n">
-        <x:v>4649.9</x:v>
+        <x:v>4689.6</x:v>
       </x:c>
       <x:c r="K2" s="12" t="n">
-        <x:v>2.4999999999999996</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="L2" s="12" t="n">
         <x:v>34.4</x:v>
       </x:c>
       <x:c r="M2" s="12" t="n">
-        <x:v>632.6</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="N2" s="12" t="n">
-        <x:v>4.8</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="O2" s="12" t="n">
-        <x:v>12.09</x:v>
+        <x:v>12.24</x:v>
       </x:c>
       <x:c r="P2" s="12" t="n">
         <x:v>1636.7</x:v>
       </x:c>
       <x:c r="Q2" s="12" t="n">
-        <x:v>2610.71</x:v>
+        <x:v>2610.79</x:v>
       </x:c>
       <x:c r="R2" s="12" t="n">
-        <x:v>261.38</x:v>
+        <x:v>261.4</x:v>
       </x:c>
       <x:c r="S2" s="12" t="n">
-        <x:v>4.4399999999999995</x:v>
+        <x:v>4.48</x:v>
       </x:c>
       <x:c r="T2" s="12" t="n">
-        <x:v>215.79999999999998</x:v>
+        <x:v>215.67</x:v>
       </x:c>
       <x:c r="U2" s="12" t="n">
-        <x:v>2.05</x:v>
+        <x:v>2.07</x:v>
       </x:c>
       <x:c r="V2" s="12" t="n">
-        <x:v>2.93</x:v>
+        <x:v>2.94</x:v>
       </x:c>
       <x:c r="W2" s="12" t="n">
-        <x:v>44.709999999999994</x:v>
+        <x:v>45.17</x:v>
       </x:c>
       <x:c r="X2" s="12" t="n">
-        <x:v>11.35</x:v>
+        <x:v>11.37</x:v>
       </x:c>
       <x:c r="Y2" s="12" t="n">
-        <x:v>3.12</x:v>
+        <x:v>3.14</x:v>
       </x:c>
       <x:c r="Z2" s="12" t="n">
-        <x:v>67.87</x:v>
+        <x:v>68.11</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4697,79 +4895,79 @@
         <x:v>Day 2</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
-        <x:v>1811.9</x:v>
+        <x:v>1810.9</x:v>
       </x:c>
       <x:c r="C3" s="12" t="n">
-        <x:v>123.6</x:v>
+        <x:v>124.3</x:v>
       </x:c>
       <x:c r="D3" s="12" t="n">
-        <x:v>233.20000000000002</x:v>
+        <x:v>232.5</x:v>
       </x:c>
       <x:c r="E3" s="12" t="n">
-        <x:v>48.1</x:v>
+        <x:v>47.7</x:v>
       </x:c>
       <x:c r="F3" s="12" t="n">
-        <x:v>46.900000000000006</x:v>
+        <x:v>46.9</x:v>
       </x:c>
       <x:c r="G3" s="12" t="n">
-        <x:v>1316.9</x:v>
+        <x:v>1271.7</x:v>
       </x:c>
       <x:c r="H3" s="12" t="n">
-        <x:v>22.299999999999997</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I3" s="12" t="n">
-        <x:v>555.3</x:v>
+        <x:v>572.8</x:v>
       </x:c>
       <x:c r="J3" s="12" t="n">
-        <x:v>5162.700000000001</x:v>
+        <x:v>5199.3</x:v>
       </x:c>
       <x:c r="K3" s="12" t="n">
         <x:v>3.2</x:v>
       </x:c>
       <x:c r="L3" s="12" t="n">
-        <x:v>6.999999999999999</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="M3" s="12" t="n">
-        <x:v>885.1999999999999</x:v>
+        <x:v>885.8</x:v>
       </x:c>
       <x:c r="N3" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="O3" s="12" t="n">
-        <x:v>11.16</x:v>
+        <x:v>11.04</x:v>
       </x:c>
       <x:c r="P3" s="12" t="n">
         <x:v>383</x:v>
       </x:c>
       <x:c r="Q3" s="12" t="n">
-        <x:v>1279.65</x:v>
+        <x:v>1279.7</x:v>
       </x:c>
       <x:c r="R3" s="12" t="n">
-        <x:v>289.74</x:v>
+        <x:v>289.77000000000004</x:v>
       </x:c>
       <x:c r="S3" s="12" t="n">
-        <x:v>7.15</x:v>
+        <x:v>7.18</x:v>
       </x:c>
       <x:c r="T3" s="12" t="n">
         <x:v>274.89</x:v>
       </x:c>
       <x:c r="U3" s="12" t="n">
-        <x:v>1.9000000000000001</x:v>
+        <x:v>1.9200000000000002</x:v>
       </x:c>
       <x:c r="V3" s="12" t="n">
         <x:v>3.6300000000000003</x:v>
       </x:c>
       <x:c r="W3" s="12" t="n">
-        <x:v>28.89</x:v>
+        <x:v>29.12</x:v>
       </x:c>
       <x:c r="X3" s="12" t="n">
-        <x:v>11.24</x:v>
+        <x:v>11.290000000000001</x:v>
       </x:c>
       <x:c r="Y3" s="12" t="n">
-        <x:v>2.91</x:v>
+        <x:v>2.9000000000000004</x:v>
       </x:c>
       <x:c r="Z3" s="12" t="n">
-        <x:v>74.8</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4777,79 +4975,79 @@
         <x:v>Day 3</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
-        <x:v>1777.9</x:v>
+        <x:v>1779.6</x:v>
       </x:c>
       <x:c r="C4" s="12" t="n">
-        <x:v>123.89999999999999</x:v>
+        <x:v>124.3</x:v>
       </x:c>
       <x:c r="D4" s="12" t="n">
-        <x:v>227.60000000000002</x:v>
+        <x:v>221.7</x:v>
       </x:c>
       <x:c r="E4" s="12" t="n">
-        <x:v>45.5</x:v>
+        <x:v>43.7</x:v>
       </x:c>
       <x:c r="F4" s="12" t="n">
-        <x:v>45.400000000000006</x:v>
+        <x:v>48.3</x:v>
       </x:c>
       <x:c r="G4" s="12" t="n">
-        <x:v>1207.3000000000002</x:v>
+        <x:v>1177.6</x:v>
       </x:c>
       <x:c r="H4" s="12" t="n">
-        <x:v>21.1</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I4" s="12" t="n">
-        <x:v>555.3</x:v>
+        <x:v>570.2</x:v>
       </x:c>
       <x:c r="J4" s="12" t="n">
-        <x:v>4417.6</x:v>
+        <x:v>4441.1</x:v>
       </x:c>
       <x:c r="K4" s="12" t="n">
-        <x:v>3.1999999999999997</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="L4" s="12" t="n">
-        <x:v>6.999999999999999</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="M4" s="12" t="n">
-        <x:v>947.4</x:v>
+        <x:v>954.7</x:v>
       </x:c>
       <x:c r="N4" s="12" t="n">
-        <x:v>2.9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="O4" s="12" t="n">
-        <x:v>10.940000000000001</x:v>
+        <x:v>11.33</x:v>
       </x:c>
       <x:c r="P4" s="12" t="n">
         <x:v>383</x:v>
       </x:c>
       <x:c r="Q4" s="12" t="n">
-        <x:v>466.90000000000003</x:v>
+        <x:v>466.75</x:v>
       </x:c>
       <x:c r="R4" s="12" t="n">
-        <x:v>268.85</x:v>
+        <x:v>268.93</x:v>
       </x:c>
       <x:c r="S4" s="12" t="n">
-        <x:v>4.72</x:v>
+        <x:v>6.53</x:v>
       </x:c>
       <x:c r="T4" s="12" t="n">
-        <x:v>310.53</x:v>
+        <x:v>310.74</x:v>
       </x:c>
       <x:c r="U4" s="12" t="n">
         <x:v>2.25</x:v>
       </x:c>
       <x:c r="V4" s="12" t="n">
-        <x:v>3.67</x:v>
+        <x:v>3.68</x:v>
       </x:c>
       <x:c r="W4" s="12" t="n">
-        <x:v>28.619999999999997</x:v>
+        <x:v>28.77</x:v>
       </x:c>
       <x:c r="X4" s="12" t="n">
-        <x:v>11.41</x:v>
+        <x:v>11.38</x:v>
       </x:c>
       <x:c r="Y4" s="12" t="n">
-        <x:v>2.95</x:v>
+        <x:v>3.01</x:v>
       </x:c>
       <x:c r="Z4" s="12" t="n">
-        <x:v>76.75</x:v>
+        <x:v>75.65</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4857,79 +5055,79 @@
         <x:v>Day 4</x:v>
       </x:c>
       <x:c r="B5" s="12" t="n">
-        <x:v>1809.6999999999998</x:v>
+        <x:v>1808.7</x:v>
       </x:c>
       <x:c r="C5" s="12" t="n">
-        <x:v>128.89999999999998</x:v>
+        <x:v>129.2</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
-        <x:v>236.4</x:v>
+        <x:v>231.1</x:v>
       </x:c>
       <x:c r="E5" s="12" t="n">
-        <x:v>41.599999999999994</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="F5" s="12" t="n">
-        <x:v>44.4</x:v>
+        <x:v>46.7</x:v>
       </x:c>
       <x:c r="G5" s="12" t="n">
-        <x:v>1011.4999999999999</x:v>
+        <x:v>1001.8</x:v>
       </x:c>
       <x:c r="H5" s="12" t="n">
-        <x:v>19.299999999999997</x:v>
+        <x:v>19.3</x:v>
       </x:c>
       <x:c r="I5" s="12" t="n">
-        <x:v>544.1</x:v>
+        <x:v>561.6</x:v>
       </x:c>
       <x:c r="J5" s="12" t="n">
-        <x:v>4793.900000000001</x:v>
+        <x:v>4811.2</x:v>
       </x:c>
       <x:c r="K5" s="12" t="n">
-        <x:v>4.800000000000001</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="L5" s="12" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="M5" s="12" t="n">
-        <x:v>957</x:v>
+        <x:v>965</x:v>
       </x:c>
       <x:c r="N5" s="12" t="n">
-        <x:v>3.6</x:v>
+        <x:v>2.9</x:v>
       </x:c>
       <x:c r="O5" s="12" t="n">
-        <x:v>9.559999999999999</x:v>
+        <x:v>9.73</x:v>
       </x:c>
       <x:c r="P5" s="12" t="n">
         <x:v>223</x:v>
       </x:c>
       <x:c r="Q5" s="12" t="n">
-        <x:v>1218.2</x:v>
+        <x:v>1218.25</x:v>
       </x:c>
       <x:c r="R5" s="12" t="n">
-        <x:v>227.87</x:v>
+        <x:v>227.93</x:v>
       </x:c>
       <x:c r="S5" s="12" t="n">
-        <x:v>6.279999999999999</x:v>
+        <x:v>8.03</x:v>
       </x:c>
       <x:c r="T5" s="12" t="n">
-        <x:v>231.38</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="U5" s="12" t="n">
-        <x:v>2.2</x:v>
+        <x:v>2.19</x:v>
       </x:c>
       <x:c r="V5" s="12" t="n">
-        <x:v>2.66</x:v>
+        <x:v>2.67</x:v>
       </x:c>
       <x:c r="W5" s="12" t="n">
-        <x:v>35.84</x:v>
+        <x:v>36.49</x:v>
       </x:c>
       <x:c r="X5" s="12" t="n">
-        <x:v>11.1</x:v>
+        <x:v>11.05</x:v>
       </x:c>
       <x:c r="Y5" s="12" t="n">
-        <x:v>3.09</x:v>
+        <x:v>3.1500000000000004</x:v>
       </x:c>
       <x:c r="Z5" s="12" t="n">
-        <x:v>63.65</x:v>
+        <x:v>62.550000000000004</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4937,79 +5135,79 @@
         <x:v>Day 5</x:v>
       </x:c>
       <x:c r="B6" s="12" t="n">
-        <x:v>1780.6999999999998</x:v>
+        <x:v>1778.8</x:v>
       </x:c>
       <x:c r="C6" s="12" t="n">
-        <x:v>124.2</x:v>
+        <x:v>124.3</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
-        <x:v>223.70000000000002</x:v>
+        <x:v>224.2</x:v>
       </x:c>
       <x:c r="E6" s="12" t="n">
-        <x:v>45</x:v>
+        <x:v>45.2</x:v>
       </x:c>
       <x:c r="F6" s="12" t="n">
-        <x:v>47.1</x:v>
+        <x:v>46.6</x:v>
       </x:c>
       <x:c r="G6" s="12" t="n">
-        <x:v>1241</x:v>
+        <x:v>1215</x:v>
       </x:c>
       <x:c r="H6" s="12" t="n">
-        <x:v>22.3</x:v>
+        <x:v>21.9</x:v>
       </x:c>
       <x:c r="I6" s="12" t="n">
-        <x:v>516.7</x:v>
+        <x:v>512.6</x:v>
       </x:c>
       <x:c r="J6" s="12" t="n">
-        <x:v>4810.4</x:v>
+        <x:v>4798.9</x:v>
       </x:c>
       <x:c r="K6" s="12" t="n">
         <x:v>3.2</x:v>
       </x:c>
       <x:c r="L6" s="12" t="n">
-        <x:v>6.999999999999999</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="M6" s="12" t="n">
-        <x:v>863.3000000000001</x:v>
+        <x:v>867.9</x:v>
       </x:c>
       <x:c r="N6" s="12" t="n">
-        <x:v>2.1</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="O6" s="12" t="n">
-        <x:v>11.2</x:v>
+        <x:v>11.06</x:v>
       </x:c>
       <x:c r="P6" s="12" t="n">
         <x:v>383</x:v>
       </x:c>
       <x:c r="Q6" s="12" t="n">
-        <x:v>1365.2</x:v>
+        <x:v>1365.35</x:v>
       </x:c>
       <x:c r="R6" s="12" t="n">
-        <x:v>264.91</x:v>
+        <x:v>265.03000000000003</x:v>
       </x:c>
       <x:c r="S6" s="12" t="n">
-        <x:v>5.4399999999999995</x:v>
+        <x:v>7.200000000000001</x:v>
       </x:c>
       <x:c r="T6" s="12" t="n">
-        <x:v>230.83999999999997</x:v>
+        <x:v>230.62</x:v>
       </x:c>
       <x:c r="U6" s="12" t="n">
-        <x:v>2.15</x:v>
+        <x:v>2.13</x:v>
       </x:c>
       <x:c r="V6" s="12" t="n">
-        <x:v>3.6900000000000004</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="W6" s="12" t="n">
-        <x:v>29.75</x:v>
+        <x:v>30.230000000000004</x:v>
       </x:c>
       <x:c r="X6" s="12" t="n">
-        <x:v>11.29</x:v>
+        <x:v>11.32</x:v>
       </x:c>
       <x:c r="Y6" s="12" t="n">
         <x:v>3.02</x:v>
       </x:c>
       <x:c r="Z6" s="12" t="n">
-        <x:v>73.83</x:v>
+        <x:v>74.07</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5017,31 +5215,31 @@
         <x:v>Day 6</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:v>1750.3000000000002</x:v>
+        <x:v>1750.5</x:v>
       </x:c>
       <x:c r="C7" s="12" t="n">
-        <x:v>125.6</x:v>
+        <x:v>126.5</x:v>
       </x:c>
       <x:c r="D7" s="12" t="n">
-        <x:v>221.9</x:v>
+        <x:v>215.5</x:v>
       </x:c>
       <x:c r="E7" s="12" t="n">
-        <x:v>46</x:v>
+        <x:v>43.9</x:v>
       </x:c>
       <x:c r="F7" s="12" t="n">
-        <x:v>45.3</x:v>
+        <x:v>48.1</x:v>
       </x:c>
       <x:c r="G7" s="12" t="n">
-        <x:v>1348.2</x:v>
+        <x:v>1318.1</x:v>
       </x:c>
       <x:c r="H7" s="12" t="n">
-        <x:v>21.5</x:v>
+        <x:v>21.6</x:v>
       </x:c>
       <x:c r="I7" s="12" t="n">
-        <x:v>584.5999999999999</x:v>
+        <x:v>618.3</x:v>
       </x:c>
       <x:c r="J7" s="12" t="n">
-        <x:v>4898.299999999999</x:v>
+        <x:v>4949.6</x:v>
       </x:c>
       <x:c r="K7" s="12" t="n">
         <x:v>5.8</x:v>
@@ -5050,46 +5248,46 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="M7" s="12" t="n">
-        <x:v>906.3</x:v>
+        <x:v>907.8</x:v>
       </x:c>
       <x:c r="N7" s="12" t="n">
-        <x:v>3.3</x:v>
+        <x:v>2.8</x:v>
       </x:c>
       <x:c r="O7" s="12" t="n">
-        <x:v>10.240000000000002</x:v>
+        <x:v>10.64</x:v>
       </x:c>
       <x:c r="P7" s="12" t="n">
         <x:v>307.8</x:v>
       </x:c>
       <x:c r="Q7" s="12" t="n">
-        <x:v>1205.5</x:v>
+        <x:v>1205.4</x:v>
       </x:c>
       <x:c r="R7" s="12" t="n">
-        <x:v>289.16</x:v>
+        <x:v>289.2</x:v>
       </x:c>
       <x:c r="S7" s="12" t="n">
-        <x:v>7.31</x:v>
+        <x:v>7.3999999999999995</x:v>
       </x:c>
       <x:c r="T7" s="12" t="n">
-        <x:v>270.36</x:v>
+        <x:v>270.57</x:v>
       </x:c>
       <x:c r="U7" s="12" t="n">
-        <x:v>2.12</x:v>
+        <x:v>2.1100000000000003</x:v>
       </x:c>
       <x:c r="V7" s="12" t="n">
         <x:v>2.69</x:v>
       </x:c>
       <x:c r="W7" s="12" t="n">
-        <x:v>32.93</x:v>
+        <x:v>33.120000000000005</x:v>
       </x:c>
       <x:c r="X7" s="12" t="n">
-        <x:v>11.719999999999999</x:v>
+        <x:v>11.68</x:v>
       </x:c>
       <x:c r="Y7" s="12" t="n">
-        <x:v>2.9699999999999998</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="Z7" s="12" t="n">
-        <x:v>74.74</x:v>
+        <x:v>73.59</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5097,133 +5295,109 @@
         <x:v>Day 7</x:v>
       </x:c>
       <x:c r="B8" s="12" t="n">
-        <x:v>1753.5</x:v>
+        <x:v>1753.1</x:v>
       </x:c>
       <x:c r="C8" s="12" t="n">
-        <x:v>122.7</x:v>
+        <x:v>122.5</x:v>
       </x:c>
       <x:c r="D8" s="12" t="n">
-        <x:v>236.6</x:v>
+        <x:v>233.6</x:v>
       </x:c>
       <x:c r="E8" s="12" t="n">
         <x:v>42.4</x:v>
       </x:c>
       <x:c r="F8" s="12" t="n">
-        <x:v>40.5</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G8" s="12" t="n">
-        <x:v>1004.5999999999999</x:v>
+        <x:v>1023.5</x:v>
       </x:c>
       <x:c r="H8" s="12" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I8" s="12" t="n">
-        <x:v>529.5</x:v>
+        <x:v>530.5</x:v>
       </x:c>
       <x:c r="J8" s="12" t="n">
-        <x:v>4985.1</x:v>
+        <x:v>4967</x:v>
       </x:c>
       <x:c r="K8" s="12" t="n">
         <x:v>3.3</x:v>
       </x:c>
       <x:c r="L8" s="12" t="n">
-        <x:v>4.8999999999999995</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="M8" s="12" t="n">
-        <x:v>852.9</x:v>
+        <x:v>858.4</x:v>
       </x:c>
       <x:c r="N8" s="12" t="n">
-        <x:v>3.4</x:v>
+        <x:v>3.1</x:v>
       </x:c>
       <x:c r="O8" s="12" t="n">
-        <x:v>9.02</x:v>
+        <x:v>9.14</x:v>
       </x:c>
       <x:c r="P8" s="12" t="n">
         <x:v>223</x:v>
       </x:c>
       <x:c r="Q8" s="12" t="n">
-        <x:v>303.1</x:v>
+        <x:v>303.25</x:v>
       </x:c>
       <x:c r="R8" s="12" t="n">
-        <x:v>277.78000000000003</x:v>
+        <x:v>277.90000000000003</x:v>
       </x:c>
       <x:c r="S8" s="12" t="n">
-        <x:v>3.92</x:v>
+        <x:v>5.66</x:v>
       </x:c>
       <x:c r="T8" s="12" t="n">
-        <x:v>331.49</x:v>
+        <x:v>331.13</x:v>
       </x:c>
       <x:c r="U8" s="12" t="n">
-        <x:v>2.36</x:v>
+        <x:v>2.33</x:v>
       </x:c>
       <x:c r="V8" s="12" t="n">
-        <x:v>3.1</x:v>
+        <x:v>3.1100000000000003</x:v>
       </x:c>
       <x:c r="W8" s="12" t="n">
-        <x:v>31.419999999999998</x:v>
+        <x:v>32.06</x:v>
       </x:c>
       <x:c r="X8" s="12" t="n">
-        <x:v>10.9</x:v>
+        <x:v>10.83</x:v>
       </x:c>
       <x:c r="Y8" s="12" t="n">
-        <x:v>3.4699999999999998</x:v>
+        <x:v>3.51</x:v>
       </x:c>
       <x:c r="Z8" s="12" t="n">
-        <x:v>51</x:v>
+        <x:v>49.949999999999996</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="28" t="str">
-        <x:v>How to read this sheet</x:v>
-      </x:c>
-      <x:c r="B10" s="28" t="str">
-        <x:v>Details</x:v>
-      </x:c>
+      <x:c r="A10" s="28"/>
+      <x:c r="B10" s="28"/>
       <x:c r="C10" s="28"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="12" t="str">
-        <x:v>Purpose</x:v>
-      </x:c>
-      <x:c r="B11" s="12" t="str">
-        <x:v>Reference only - these values mirror the final meal plan and do not change shopping quantities.</x:v>
-      </x:c>
+      <x:c r="A11" s="12"/>
+      <x:c r="B11" s="12"/>
       <x:c r="C11" s="12"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="12" t="str">
-        <x:v>Vitamin E/K note</x:v>
-      </x:c>
-      <x:c r="B12" s="12" t="str">
-        <x:v>Cooking-oil contribution is excluded because the exact oil type is unspecified.</x:v>
-      </x:c>
+      <x:c r="A12" s="12"/>
+      <x:c r="B12" s="12"/>
       <x:c r="C12" s="12"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="12" t="str">
-        <x:v>Biotin note</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="str">
-        <x:v>Vitamin B7/biotin is an estimate; generic food datasets often have incomplete biotin data.</x:v>
-      </x:c>
+      <x:c r="A13" s="12"/>
+      <x:c r="B13" s="12"/>
       <x:c r="C13" s="12"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="12" t="str">
-        <x:v>Vitamin D note</x:v>
-      </x:c>
-      <x:c r="B14" s="12" t="str">
-        <x:v>Most days remain below the 15 µg/day food target; this is intentionally not corrected by increasing cod liver.</x:v>
-      </x:c>
+      <x:c r="A14" s="12"/>
+      <x:c r="B14" s="12"/>
       <x:c r="C14" s="12"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="12" t="str">
-        <x:v>Source basis</x:v>
-      </x:c>
-      <x:c r="B15" s="12" t="str">
-        <x:v>Generic food-composition planning estimates synchronized from the final meal-plan workbook.</x:v>
-      </x:c>
+      <x:c r="A15" s="12"/>
+      <x:c r="B15" s="12"/>
       <x:c r="C15" s="12"/>
     </x:row>
   </x:sheetData>
@@ -5379,18 +5553,18 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="78" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="85" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="31" t="str">
+      <x:c r="A1" s="46" t="str">
         <x:v>Nutrient</x:v>
       </x:c>
-      <x:c r="B1" s="31" t="str">
+      <x:c r="B1" s="46" t="str">
         <x:v>Target / guide</x:v>
       </x:c>
-      <x:c r="C1" s="31" t="str">
+      <x:c r="C1" s="46" t="str">
         <x:v>Interpretation</x:v>
       </x:c>
     </x:row>
@@ -5523,7 +5697,7 @@
         <x:v>15 mg/day</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>Adult RDA. Cooking-oil vitamin E is excluded because the specific oil was not defined, so totals are conservative.</x:v>
+        <x:v>Adult RDA. The new sunflower-seed rotation raises food Vitamin E, but generic totals remain below 15 mg/day; unspecified cooking oil is still excluded and could materially change the total.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -5650,4 +5824,1151 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="37" t="str">
+        <x:v>Day</x:v>
+      </x:c>
+      <x:c r="B1" s="37" t="str">
+        <x:v>Option</x:v>
+      </x:c>
+      <x:c r="C1" s="37" t="str">
+        <x:v>Breakfast</x:v>
+      </x:c>
+      <x:c r="D1" s="37" t="str">
+        <x:v>Key grains / legumes</x:v>
+      </x:c>
+      <x:c r="E1" s="37" t="str">
+        <x:v>Seed side</x:v>
+      </x:c>
+      <x:c r="F1" s="37" t="str">
+        <x:v>Milk</x:v>
+      </x:c>
+      <x:c r="G1" s="37" t="str">
+        <x:v>Eggs / egg whites</x:v>
+      </x:c>
+      <x:c r="H1" s="37" t="str">
+        <x:v>Shopping note</x:v>
+      </x:c>
+      <x:c r="I1" s="37" t="str">
+        <x:v>Morning effort</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="12" t="str">
+        <x:v>Day 1</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="str">
+        <x:v>Warm Oats + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="str">
+        <x:v>Oats 45 g</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="str">
+        <x:v>Chia seeds 8 g
+Ground flaxseed 7 g
+Hemp hearts 5 g</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G2" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 100 g</x:v>
+      </x:c>
+      <x:c r="H2" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I2" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="12" t="str">
+        <x:v>Day 1</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="str">
+        <x:v>Chia seeds 8 g
+Ground flaxseed 7 g
+Hemp hearts 5 g</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G3" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H3" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I3" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="12" t="str">
+        <x:v>Day 1</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="str">
+        <x:v>Chia seeds 8 g
+Ground flaxseed 7 g
+Hemp hearts 5 g</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="str">
+        <x:v>Low-fat milk 285 ml</x:v>
+      </x:c>
+      <x:c r="G4" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H4" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I4" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="12" t="str">
+        <x:v>Day 1</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="str">
+        <x:v>Rolled oats 40 g
+Ready-to-eat / steam-processed ragi flakes 10 g</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="str">
+        <x:v>Chia seeds 8 g
+Ground flaxseed 7 g
+Hemp hearts 5 g</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G5" s="12" t="str">
+        <x:v>Whole eggs 1
+Batch-cooked egg whites 100 g</x:v>
+      </x:c>
+      <x:c r="H5" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="12" t="str">
+        <x:v>Day 2</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>Ragi Milk Porridge + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="str">
+        <x:v>Ragi flour 45 g</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Hemp hearts 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G6" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H6" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="12" t="str">
+        <x:v>Day 2</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Hemp hearts 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G7" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H7" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I7" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="12" t="str">
+        <x:v>Day 2</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Hemp hearts 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G8" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H8" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I8" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="12" t="str">
+        <x:v>Day 2</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="str">
+        <x:v>Ready-to-eat / steam-processed ragi flakes 45 g</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Hemp hearts 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G9" s="12" t="str">
+        <x:v>Whole eggs 1
+Batch-cooked egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H9" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I9" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="str">
+        <x:v>Day 3</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
+        <x:v>Warm Oats + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="str">
+        <x:v>Oats 37 g</x:v>
+      </x:c>
+      <x:c r="E10" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Pumpkin seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F10" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G10" s="12" t="str">
+        <x:v>Whole eggs 2
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H10" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I10" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="str">
+        <x:v>Day 3</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D11" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Pumpkin seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F11" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G11" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H11" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I11" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="str">
+        <x:v>Day 3</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D12" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Pumpkin seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G12" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H12" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I12" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="12" t="str">
+        <x:v>Day 3</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="str">
+        <x:v>Rolled oats 35 g
+Ready-to-eat / steam-processed ragi flakes 15 g</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Pumpkin seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G13" s="12" t="str">
+        <x:v>Whole eggs 2
+Batch-cooked egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H13" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I13" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="12" t="str">
+        <x:v>Day 4</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
+        <x:v>Warm Oats + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="str">
+        <x:v>Oats 37 g</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Hemp hearts 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G14" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H14" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I14" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="12" t="str">
+        <x:v>Day 4</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Hemp hearts 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G15" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 35 g</x:v>
+      </x:c>
+      <x:c r="H15" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I15" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="12" t="str">
+        <x:v>Day 4</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Hemp hearts 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G16" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 15 g</x:v>
+      </x:c>
+      <x:c r="H16" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I16" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="12" t="str">
+        <x:v>Day 4</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="str">
+        <x:v>Ready-to-eat / steam-processed ragi flakes 10 g
+Thick poha / flattened rice 40 g</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Hemp hearts 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G17" s="12" t="str">
+        <x:v>Whole eggs 1
+Batch-cooked egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H17" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I17" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="12" t="str">
+        <x:v>Day 5</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>Ragi Milk Porridge + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>Ragi flour 45 g</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Sunflower seeds 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G18" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H18" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I18" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="12" t="str">
+        <x:v>Day 5</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Sunflower seeds 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G19" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H19" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I19" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="12" t="str">
+        <x:v>Day 5</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Sunflower seeds 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G20" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H20" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I20" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="12" t="str">
+        <x:v>Day 5</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="str">
+        <x:v>Rolled oats 15 g
+Ready-to-eat / steam-processed ragi flakes 35 g</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="str">
+        <x:v>Sesame seeds 5 g
+Sunflower seeds 5 g
+Chia seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G21" s="12" t="str">
+        <x:v>Whole eggs 1
+Batch-cooked egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H21" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I21" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="12" t="str">
+        <x:v>Day 6</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="12" t="str">
+        <x:v>Warm Oats + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D22" s="12" t="str">
+        <x:v>Oats 37 g</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Hemp hearts 5 g
+Pumpkin seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F22" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G22" s="12" t="str">
+        <x:v>Whole eggs 2</x:v>
+      </x:c>
+      <x:c r="H22" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I22" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="12" t="str">
+        <x:v>Day 6</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C23" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D23" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E23" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Hemp hearts 5 g
+Pumpkin seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F23" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G23" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H23" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I23" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="12" t="str">
+        <x:v>Day 6</x:v>
+      </x:c>
+      <x:c r="B24" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C24" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D24" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E24" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Hemp hearts 5 g
+Pumpkin seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F24" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G24" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H24" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I24" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="12" t="str">
+        <x:v>Day 6</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C25" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D25" s="12" t="str">
+        <x:v>Ready-to-eat / steam-processed ragi flakes 20 g
+Thick poha / flattened rice 30 g</x:v>
+      </x:c>
+      <x:c r="E25" s="12" t="str">
+        <x:v>Chia seeds 5 g
+Hemp hearts 5 g
+Pumpkin seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F25" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G25" s="12" t="str">
+        <x:v>Whole eggs 2</x:v>
+      </x:c>
+      <x:c r="H25" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I25" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="12" t="str">
+        <x:v>Day 7</x:v>
+      </x:c>
+      <x:c r="B26" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C26" s="12" t="str">
+        <x:v>Warm Oats + Eggs + Separate Seed Side</x:v>
+      </x:c>
+      <x:c r="D26" s="12" t="str">
+        <x:v>Oats 38 g</x:v>
+      </x:c>
+      <x:c r="E26" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Chia seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F26" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G26" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 100 g</x:v>
+      </x:c>
+      <x:c r="H26" s="12" t="str">
+        <x:v>Base recommended shopping plan. Main Store Comparison quantities are calculated from Option 1 across all 7 days.</x:v>
+      </x:c>
+      <x:c r="I26" s="12" t="str">
+        <x:v>Cook grain/eggs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="12" t="str">
+        <x:v>Day 7</x:v>
+      </x:c>
+      <x:c r="B27" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C27" s="12" t="str">
+        <x:v>Unsalted Ragi-Moong Chilla + Milk + Egg</x:v>
+      </x:c>
+      <x:c r="D27" s="12" t="str">
+        <x:v>Ragi flour 25 g
+Moong dal (dry) 25 g</x:v>
+      </x:c>
+      <x:c r="E27" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Chia seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F27" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G27" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H27" s="12" t="str">
+        <x:v>Optional cooked variety. Buy extra ragi/moong only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I27" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="12" t="str">
+        <x:v>Day 7</x:v>
+      </x:c>
+      <x:c r="B28" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C28" s="12" t="str">
+        <x:v>Unsalted Poha-Moong Egg Bowl + Milk</x:v>
+      </x:c>
+      <x:c r="D28" s="12" t="str">
+        <x:v>Thick poha / flattened rice (dry) 25 g
+Moong dal (dry) 20 g
+Frozen sweet peas [CF] 50 g</x:v>
+      </x:c>
+      <x:c r="E28" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Chia seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F28" s="12" t="str">
+        <x:v>Low-fat milk 275 ml</x:v>
+      </x:c>
+      <x:c r="G28" s="12" t="str">
+        <x:v>Whole eggs 1
+Egg whites 50 g</x:v>
+      </x:c>
+      <x:c r="H28" s="12" t="str">
+        <x:v>Optional poha-moong variety. Buy poha/moong/peas only on days you choose this option.</x:v>
+      </x:c>
+      <x:c r="I28" s="12" t="str">
+        <x:v>6–10 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="12" t="str">
+        <x:v>Day 7</x:v>
+      </x:c>
+      <x:c r="B29" s="12" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C29" s="12" t="str">
+        <x:v>Overnight No-Cook Breakfast Jar + Pre-Cooked Eggs</x:v>
+      </x:c>
+      <x:c r="D29" s="12" t="str">
+        <x:v>Rolled oats 30 g
+Ready-to-eat / steam-processed ragi flakes 20 g</x:v>
+      </x:c>
+      <x:c r="E29" s="12" t="str">
+        <x:v>Ground flaxseed 5 g
+Chia seeds 5 g
+Sunflower seeds 5 g</x:v>
+      </x:c>
+      <x:c r="F29" s="12" t="str">
+        <x:v>Low-fat milk 300 ml</x:v>
+      </x:c>
+      <x:c r="G29" s="12" t="str">
+        <x:v>Whole eggs 1
+Batch-cooked egg whites 100 g</x:v>
+      </x:c>
+      <x:c r="H29" s="12" t="str">
+        <x:v>Overnight no-cook morning option. Buy ready-to-eat/steam-processed ragi flakes where listed; do not substitute raw ragi flour.</x:v>
+      </x:c>
+      <x:c r="I29" s="12" t="str">
+        <x:v>0 min cooking</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="43" t="str">
+        <x:v>If choosing Overnight Option 4 every day</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str"/>
+      <x:c r="C32" s="12" t="str"/>
+      <x:c r="D32" s="12" t="str"/>
+      <x:c r="E32" s="12" t="str"/>
+      <x:c r="F32" s="12" t="str"/>
+      <x:c r="G32" s="12"/>
+      <x:c r="H32" s="12"/>
+      <x:c r="I32" s="12"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="44" t="str">
+        <x:v>Ingredient</x:v>
+      </x:c>
+      <x:c r="B33" s="44" t="str">
+        <x:v>Weekly amount</x:v>
+      </x:c>
+      <x:c r="C33" s="44" t="str">
+        <x:v>Where to look</x:v>
+      </x:c>
+      <x:c r="D33" s="44" t="str">
+        <x:v>Why</x:v>
+      </x:c>
+      <x:c r="E33" s="44" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+      <x:c r="F33" s="44" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="G33" s="12"/>
+      <x:c r="H33" s="12"/>
+      <x:c r="I33" s="12"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="12" t="str">
+        <x:v>Rolled oats</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>120 g</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str">
+        <x:v>Walmart / Costco</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="str">
+        <x:v>Used on Days 1, 3, 5, 7</x:v>
+      </x:c>
+      <x:c r="E34" s="12" t="str">
+        <x:v>Rolled oats can soak overnight in milk.</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="str">
+        <x:v>Optional</x:v>
+      </x:c>
+      <x:c r="G34" s="12"/>
+      <x:c r="H34" s="12"/>
+      <x:c r="I34" s="12"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="12" t="str">
+        <x:v>RTE / steam-processed ragi flakes</x:v>
+      </x:c>
+      <x:c r="B35" s="12" t="str">
+        <x:v>155 g</x:v>
+      </x:c>
+      <x:c r="C35" s="12" t="str">
+        <x:v>Lotte / Indian grocery</x:v>
+      </x:c>
+      <x:c r="D35" s="12" t="str">
+        <x:v>Used across several overnight jars</x:v>
+      </x:c>
+      <x:c r="E35" s="12" t="str">
+        <x:v>Use label-confirmed ready-to-eat or steam-processed flakes; not raw flour.</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="str">
+        <x:v>Optional</x:v>
+      </x:c>
+      <x:c r="G35" s="12"/>
+      <x:c r="H35" s="12"/>
+      <x:c r="I35" s="12"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="12" t="str">
+        <x:v>Thick poha / flattened rice</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
+        <x:v>40 g</x:v>
+      </x:c>
+      <x:c r="C36" s="12" t="str">
+        <x:v>Lotte / Indian grocery</x:v>
+      </x:c>
+      <x:c r="D36" s="12" t="str">
+        <x:v>Day 4 overnight jar</x:v>
+      </x:c>
+      <x:c r="E36" s="12" t="str">
+        <x:v>Use plain thick poha; refrigerate overnight.</x:v>
+      </x:c>
+      <x:c r="F36" s="12" t="str">
+        <x:v>Optional</x:v>
+      </x:c>
+      <x:c r="G36" s="12"/>
+      <x:c r="H36" s="12"/>
+      <x:c r="I36" s="12"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="12" t="str">
+        <x:v>Low-fat milk</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>2,100 ml</x:v>
+      </x:c>
+      <x:c r="C37" s="12" t="str">
+        <x:v>Walmart</x:v>
+      </x:c>
+      <x:c r="D37" s="12" t="str">
+        <x:v>Same weekly amount as base plan</x:v>
+      </x:c>
+      <x:c r="E37" s="12" t="str">
+        <x:v>No additional milk needed if replacing Option 1.</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
+        <x:v>Same total</x:v>
+      </x:c>
+      <x:c r="G37" s="12"/>
+      <x:c r="H37" s="12"/>
+      <x:c r="I37" s="12"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="12" t="str">
+        <x:v>Whole eggs</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>9 breakfast eggs</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str">
+        <x:v>Walmart</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="str">
+        <x:v>Same breakfast count as base plan</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="str">
+        <x:v>Batch-cook in advance.</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>Same total</x:v>
+      </x:c>
+      <x:c r="G38" s="12"/>
+      <x:c r="H38" s="12"/>
+      <x:c r="I38" s="12"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="12" t="str">
+        <x:v>Egg whites</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>400 g breakfast egg whites</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="str">
+        <x:v>Walmart</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="str">
+        <x:v>Same breakfast amount as base plan</x:v>
+      </x:c>
+      <x:c r="E39" s="12" t="str">
+        <x:v>Batch-cook/portion in advance.</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
+        <x:v>Same total</x:v>
+      </x:c>
+      <x:c r="G39" s="12"/>
+      <x:c r="H39" s="12"/>
+      <x:c r="I39" s="12"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A32:F32"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>